<commit_message>
Add Automatic Ordering procurement context
</commit_message>
<xml_diff>
--- a/outputs/vendor_invoice_autopilot_workbook.xlsx
+++ b/outputs/vendor_invoice_autopilot_workbook.xlsx
@@ -8,9 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vendors" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="purchase_orders" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="invoice_reviews" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="demo_reviews_backup" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="demand_forecasts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inventory_position" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="supplier_rules" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="purchase_orders" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="invoice_reviews" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="demo_reviews_backup" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -554,6 +557,440 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>forecast_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>vendor_name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>forecast_period</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>forecast_quantity</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>required_by</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>business_reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FC-2026-ACME-Q2-PACKAGING</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Packaging materials</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Acme Packaging</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-Q2</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.91</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Q2 outbound packaging demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FC-2026-POS-JUNE-OFFICE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Office paper and toner</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Prague Office Supplies</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.86</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>June office supplies replenishment</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>current_stock</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>reorder_point</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>safety_stock</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>open_po_quantity</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>projected_stockout_date</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>warehouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Packaging materials</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Prague DC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Office paper and toner</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Prague HQ</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>vendor_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>approved_po_prefix</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>max_auto_po_amount</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>lead_time_days</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>requires_finance_approval_over</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>preferred_terms_days</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Acme Packaging</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PO-2026-ACME</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Prague Office Supplies</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PO-2026-POS</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -698,7 +1135,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -812,7 +1249,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>